<commit_message>
Use green text for BYH OA additions
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -69,8 +69,12 @@
       <b val="1"/>
       <color rgb="0017365D"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -87,8 +91,13 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -154,11 +163,25 @@
         <color rgb="00E1E7EC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2EC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E2EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -189,6 +212,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6358,7 +6396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.75" customWidth="1" min="1" max="1"/>
@@ -6372,7 +6410,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -6478,6 +6515,18 @@
       <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Do not renumber or delete sections by default. Track any affected Section / Article / Exhibit references on the Reference Audit tab before a build is review-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Drafting Colors</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Jeff red edits remain red source text; future BYH additions/replacements use green font and are tracked by source class.</t>
         </is>
       </c>
     </row>
@@ -12577,7 +12626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z203"/>
+  <dimension ref="A1:Z206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12851,7 +12900,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Do not delete unwanted source text; use strikethrough and add replacement text in red.</t>
+          <t>Do not delete unwanted source text; use strikethrough and add replacement text in green.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -13091,7 +13140,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Preserve source run formatting for unchanged and struck source text. Added BYH text is red but otherwise matches surrounding formatting.</t>
+          <t>Preserve source run formatting for unchanged and struck source text. Added BYH text is green but otherwise matches surrounding formatting.</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -18748,6 +18797,132 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="14" t="inlineStr">
+        <is>
+          <t>R-018</t>
+        </is>
+      </c>
+      <c r="B204" s="14" t="inlineStr">
+        <is>
+          <t>Source Color Preservation</t>
+        </is>
+      </c>
+      <c r="C204" s="14" t="inlineStr">
+        <is>
+          <t>Preserve Jeff Watson's later review edits as red-font source text. Do not recolor Jeff's red edits in BYH derivative builds.</t>
+        </is>
+      </c>
+      <c r="D204" s="14" t="inlineStr">
+        <is>
+          <t>All future builds</t>
+        </is>
+      </c>
+      <c r="E204" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F204" s="14" t="inlineStr">
+        <is>
+          <t>Maintains Jeff/Codex authorship distinction</t>
+        </is>
+      </c>
+      <c r="G204" s="14" t="inlineStr">
+        <is>
+          <t>Visual spot-check red text source class</t>
+        </is>
+      </c>
+      <c r="H204" s="14" t="inlineStr">
+        <is>
+          <t>Wes approved Codex recommendation on 2026-06-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="14" t="inlineStr">
+        <is>
+          <t>R-019</t>
+        </is>
+      </c>
+      <c r="B205" s="14" t="inlineStr">
+        <is>
+          <t>BYH Addition Color</t>
+        </is>
+      </c>
+      <c r="C205" s="14" t="inlineStr">
+        <is>
+          <t>Use green font for new BYH additions and replacement text going forward, while otherwise matching surrounding source formatting unless Wes gives a different style instruction.</t>
+        </is>
+      </c>
+      <c r="D205" s="14" t="inlineStr">
+        <is>
+          <t>BYH builds</t>
+        </is>
+      </c>
+      <c r="E205" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F205" s="14" t="inlineStr">
+        <is>
+          <t>Distinguishes BYH additions from Jeff red source edits</t>
+        </is>
+      </c>
+      <c r="G205" s="14" t="inlineStr">
+        <is>
+          <t>Visual spot-check green additions</t>
+        </is>
+      </c>
+      <c r="H205" s="14" t="inlineStr">
+        <is>
+          <t>Future builds only unless Wes asks to retrofit prior versions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="14" t="inlineStr">
+        <is>
+          <t>R-020</t>
+        </is>
+      </c>
+      <c r="B206" s="14" t="inlineStr">
+        <is>
+          <t>Change Source Tracking</t>
+        </is>
+      </c>
+      <c r="C206" s="14" t="inlineStr">
+        <is>
+          <t>Record the author/source class for visible drafting changes, including Jeff source edit, Wes simplified text, BYH addition, and BYH strikeout.</t>
+        </is>
+      </c>
+      <c r="D206" s="14" t="inlineStr">
+        <is>
+          <t>Article Map and Reference Audit</t>
+        </is>
+      </c>
+      <c r="E206" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F206" s="14" t="inlineStr">
+        <is>
+          <t>Makes color and authorship auditable</t>
+        </is>
+      </c>
+      <c r="G206" s="14" t="inlineStr">
+        <is>
+          <t>Source Class populated where applicable</t>
+        </is>
+      </c>
+      <c r="H206" s="14" t="inlineStr">
+        <is>
+          <t>Use controlled list values.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -18773,6 +18948,8 @@
     <col width="26.25" customWidth="1" min="7" max="7"/>
     <col width="37.5" customWidth="1" min="8" max="8"/>
     <col width="16.25" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -18782,54 +18959,63 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Article / Section</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Baseline Location</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>BYH Change Needed</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Redline Treatment</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Formatting Rule</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Current Status</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>Verification</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="15" t="inlineStr">
         <is>
           <t>Open Question</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="15" t="inlineStr">
         <is>
           <t>Rule IDs</t>
         </is>
       </c>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>Source Class</t>
+        </is>
+      </c>
+      <c r="K3" s="16" t="inlineStr">
+        <is>
+          <t>Visible Color Rule</t>
+        </is>
+      </c>
       <c r="L3" s="5" t="n"/>
       <c r="M3" s="5" t="n"/>
       <c r="N3" s="5" t="n"/>
@@ -18864,7 +19050,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Strike retirement-only source text; add BYH trust language in red.</t>
+          <t>Strike retirement-only source text; add BYH trust language in green.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -18892,8 +19078,16 @@
           <t>R-004, R-008, R-012</t>
         </is>
       </c>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="n"/>
       <c r="N4" s="5" t="n"/>
@@ -18956,8 +19150,16 @@
           <t>R-006</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
@@ -19020,8 +19222,16 @@
           <t>R-005</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="5" t="n"/>
@@ -19056,7 +19266,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Add red BYH paragraph between clauses.</t>
+          <t>Add green BYH paragraph between clauses.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -19084,8 +19294,16 @@
           <t>R-006, R-007, R-012</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
@@ -19148,8 +19366,16 @@
           <t>R-004, R-010</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="n"/>
       <c r="N8" s="5" t="n"/>
@@ -19184,12 +19410,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Inline strike/replacement redline.</t>
+          <t>Inline strike/replacement greenline.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Preserve blue/bold/11-point source formatting; red text matches except color.</t>
+          <t>Preserve blue/bold/11-point source formatting; green text matches except color.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -19212,8 +19438,16 @@
           <t>R-008, R-012</t>
         </is>
       </c>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L9" s="5" t="n"/>
       <c r="M9" s="5" t="n"/>
       <c r="N9" s="5" t="n"/>
@@ -19276,8 +19510,16 @@
           <t>R-008, R-009, R-011</t>
         </is>
       </c>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="n"/>
@@ -19340,8 +19582,16 @@
           <t>R-004, R-005</t>
         </is>
       </c>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L11" s="5" t="n"/>
       <c r="M11" s="5" t="n"/>
       <c r="N11" s="5" t="n"/>
@@ -19404,8 +19654,16 @@
           <t>R-011</t>
         </is>
       </c>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
@@ -19440,7 +19698,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Strike contradictory heading/text; insert red replacement.</t>
+          <t>Strike contradictory heading/text; insert green replacement.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -19468,8 +19726,16 @@
           <t>R-013</t>
         </is>
       </c>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L13" s="5" t="n"/>
       <c r="M13" s="5" t="n"/>
       <c r="N13" s="5" t="n"/>
@@ -19504,7 +19770,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Strike retirement-account signature language; add BYH blocks in red.</t>
+          <t>Strike retirement-account signature language; add BYH blocks in green.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -19532,8 +19798,16 @@
           <t>R-011, R-012</t>
         </is>
       </c>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="n"/>
       <c r="N14" s="5" t="n"/>
@@ -19568,7 +19842,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Strike prior retirement member table; add BYH table/rows in red.</t>
+          <t>Strike prior retirement member table; add BYH table/rows in green.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -19596,8 +19870,16 @@
           <t>R-012</t>
         </is>
       </c>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>BYH addition / source strikeout as applicable</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Preserve source colors; new BYH additions/replacements green.</t>
+        </is>
+      </c>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
       <c r="N15" s="5" t="n"/>
@@ -24808,14 +25090,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57142857142857" customWidth="1" min="1" max="1"/>
     <col width="15.71428571428571" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="24.28571428571428" customWidth="1" min="4" max="4"/>
-    <col width="19.28571428571428" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="42.85714285714285" customWidth="1" min="6" max="6"/>
     <col width="42.85714285714285" customWidth="1" min="7" max="7"/>
     <col width="21.42857142857143" customWidth="1" min="8" max="8"/>
@@ -24831,52 +25113,57 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Audit ID</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Build Version</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>Changed Section / Label</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>Change Type</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>Source Class</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>Reference-Sensitive?</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>Internal References Found</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>Treatment</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="I3" s="17" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>Reviewer / Owner</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -24903,32 +25190,37 @@
           <t>New label</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>TBD during build</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>Search whole document for Section / Article / Exhibit references</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>Prefer suffix numbering or insertion inside existing section</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>Use before review-ready status.</t>
         </is>
@@ -24955,32 +25247,37 @@
           <t>Section retained with strikethrough</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>TBD during build</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Search for direct references to retained number</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>Do not delete number unless renumbering separately approved</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Preserve number to avoid broken references.</t>
         </is>
@@ -25007,32 +25304,37 @@
           <t>Relocation without renumbering</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>TBD during build</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Search old and new nearby section references</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Add language without shifting later sections where possible</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>Document why placement does not disturb references.</t>
         </is>
@@ -25059,32 +25361,37 @@
           <t>Renumbering cleanup</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>TBD during build</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Full cross-reference scan required</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>Update all affected references and comparison notes</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="J7" s="9" t="inlineStr">
         <is>
           <t>Codex / Wes</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>Only after Wes explicitly approves renumbering.</t>
         </is>
@@ -30926,7 +31233,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -36921,7 +37227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.5" customWidth="1" min="1" max="1"/>
@@ -36929,6 +37235,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="11.25" customWidth="1" min="4" max="4"/>
     <col width="18.75" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -36938,7 +37246,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -36965,6 +37272,16 @@
           <t>Phases</t>
         </is>
       </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>Change Source Class</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Visible Color Rule</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -36992,6 +37309,16 @@
           <t>Authorization</t>
         </is>
       </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Jeff source edit</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Jeff source edit = preserve red</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -37019,6 +37346,16 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Wes simplified text</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Wes simplified text = preserve blue</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -37046,6 +37383,16 @@
           <t>Inputs</t>
         </is>
       </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Jeff original text</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Jeff original text = preserve black</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -37069,6 +37416,16 @@
           <t>Build</t>
         </is>
       </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>BYH addition</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>BYH addition/replacement = green</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -37090,6 +37447,16 @@
       <c r="E8" s="1" t="inlineStr">
         <is>
           <t>QA</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>BYH replacement</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>BYH strikeout = preserve source color + strikethrough</t>
         </is>
       </c>
     </row>
@@ -37111,6 +37478,11 @@
           <t>Documentation</t>
         </is>
       </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>BYH strikeout</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -37128,6 +37500,11 @@
       <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Git</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Attorney/CPA review item</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep BYH section 5.1bxi operative
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -225,6 +225,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12626,7 +12629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z206"/>
+  <dimension ref="A1:Z207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12646,7 +12649,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -18920,6 +18922,48 @@
       <c r="H206" s="14" t="inlineStr">
         <is>
           <t>Use controlled list values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="14" t="inlineStr">
+        <is>
+          <t>R-021</t>
+        </is>
+      </c>
+      <c r="B207" s="14" t="inlineStr">
+        <is>
+          <t>BYH Article 5 Retained Clause</t>
+        </is>
+      </c>
+      <c r="C207" s="14" t="inlineStr">
+        <is>
+          <t>For BYH, Section 5.1(b)(xi) should remain operative and should not be struck. Jeff's strikeout is acceptable source history in the simplified OA, but the BYH build should restore the clause as retained text because it applies to BYH.</t>
+        </is>
+      </c>
+      <c r="D207" s="14" t="inlineStr">
+        <is>
+          <t>BYH fresh builds</t>
+        </is>
+      </c>
+      <c r="E207" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F207" s="14" t="inlineStr">
+        <is>
+          <t>Overrides Jeff strikeout for this clause in BYH output</t>
+        </is>
+      </c>
+      <c r="G207" s="14" t="inlineStr">
+        <is>
+          <t>Check 5.1(b)(xi) is not struck in review-ready BYH draft</t>
+        </is>
+      </c>
+      <c r="H207" s="14" t="inlineStr">
+        <is>
+          <t>Wes instruction on 2026-06-08.</t>
         </is>
       </c>
     </row>
@@ -18959,7 +19003,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -19609,59 +19652,59 @@
       <c r="Z11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>5.1(b)(xi)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Manager number change clause</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Keep operative for BYH.</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>No exclusion.</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Preserve source.</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Text present.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Article 5 manager powers list</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Retain this clause as operative for BYH even if Jeff struck it in the simplified OA source.</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Do not carry forward Jeff's strikeout for BYH; restore as retained source text unless Wes gives a later contrary instruction.</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Preserve the clause's surrounding list formatting and source style; do not add a replacement note.</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Rule recorded for next build</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>Confirm 5.1(b)(xi) appears unstruck in the next review-ready BYH draft.</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>None currently.</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>R-011</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>BYH addition / source strikeout as applicable</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>Preserve source colors; new BYH additions/replacements green.</t>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>R-021</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>Jeff source edit overridden for BYH applicability</t>
+        </is>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>Retained text should not be green merely because a Jeff strikeout was rejected; use green only if new BYH language is added.</t>
         </is>
       </c>
       <c r="L12" s="5" t="n"/>
@@ -31213,7 +31256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z201"/>
+  <dimension ref="A1:Z202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -31233,6 +31276,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -31574,7 +31618,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Verify unchanged/struck source formatting is preserved and BYH text is red.</t>
+          <t>Verify unchanged/struck source formatting is preserved and BYH text is green.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -37212,6 +37256,60 @@
           <t>Required before review-ready status; do not renumber by default.</t>
         </is>
       </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B202" s="14" t="inlineStr">
+        <is>
+          <t>Article 5</t>
+        </is>
+      </c>
+      <c r="C202" s="14" t="inlineStr">
+        <is>
+          <t>Confirm Section 5.1(b)(xi) remains operative and unstruck for BYH.</t>
+        </is>
+      </c>
+      <c r="D202" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E202" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F202" s="14" t="n"/>
+      <c r="G202" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H202" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-021.</t>
+        </is>
+      </c>
+      <c r="I202" s="14" t="n"/>
+      <c r="J202" s="14" t="n"/>
+      <c r="K202" s="14" t="n"/>
+      <c r="L202" s="14" t="n"/>
+      <c r="M202" s="14" t="n"/>
+      <c r="N202" s="14" t="n"/>
+      <c r="O202" s="14" t="n"/>
+      <c r="P202" s="14" t="n"/>
+      <c r="Q202" s="14" t="n"/>
+      <c r="R202" s="14" t="n"/>
+      <c r="S202" s="14" t="n"/>
+      <c r="T202" s="14" t="n"/>
+      <c r="U202" s="14" t="n"/>
+      <c r="V202" s="14" t="n"/>
+      <c r="W202" s="14" t="n"/>
+      <c r="X202" s="14" t="n"/>
+      <c r="Y202" s="14" t="n"/>
+      <c r="Z202" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add BYH opening paragraph formatting rules
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -12629,7 +12629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z207"/>
+  <dimension ref="A1:Z209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12649,6 +12649,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -18964,6 +18965,90 @@
       <c r="H207" s="14" t="inlineStr">
         <is>
           <t>Wes instruction on 2026-06-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="14" t="inlineStr">
+        <is>
+          <t>R-022</t>
+        </is>
+      </c>
+      <c r="B208" s="14" t="inlineStr">
+        <is>
+          <t>Opening Ownership Formatting</t>
+        </is>
+      </c>
+      <c r="C208" s="14" t="inlineStr">
+        <is>
+          <t>In the opening ownership block, keep the trust sentence on the first line. Put each later ownership-authority line on its own line and indent each later line by 4 characters: This sole Member acts through its co-trustees; Wesley Dale Browning and; Jeanette Wilson Hollinger, or; any successor trustee authorized under the trust documents.</t>
+        </is>
+      </c>
+      <c r="D208" s="14" t="inlineStr">
+        <is>
+          <t>BYH opening paragraphs</t>
+        </is>
+      </c>
+      <c r="E208" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F208" s="14" t="inlineStr">
+        <is>
+          <t>Controls visible opening ownership block format</t>
+        </is>
+      </c>
+      <c r="G208" s="14" t="inlineStr">
+        <is>
+          <t>Check line breaks and 4-character indent after first line</t>
+        </is>
+      </c>
+      <c r="H208" s="14" t="inlineStr">
+        <is>
+          <t>Wes instruction on 2026-06-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="14" t="inlineStr">
+        <is>
+          <t>R-023</t>
+        </is>
+      </c>
+      <c r="B209" s="14" t="inlineStr">
+        <is>
+          <t>Opening Entity Replacement Spacing</t>
+        </is>
+      </c>
+      <c r="C209" s="14" t="inlineStr">
+        <is>
+          <t>Preserve proper spacing around the opening agreement sentence entity-name replacement so the text does not join as ofSell Your Home, LLCBuy Your Home, LLC. The clean BYH reading should be: this Amended and Restated Operating Agreement of Buy Your Home, LLC.</t>
+        </is>
+      </c>
+      <c r="D209" s="14" t="inlineStr">
+        <is>
+          <t>BYH opening paragraphs</t>
+        </is>
+      </c>
+      <c r="E209" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F209" s="14" t="inlineStr">
+        <is>
+          <t>Prevents joined words around entity replacement</t>
+        </is>
+      </c>
+      <c r="G209" s="14" t="inlineStr">
+        <is>
+          <t>Search opening paragraphs for joined ofSell/LLCBuy text and confirm clean spacing</t>
+        </is>
+      </c>
+      <c r="H209" s="14" t="inlineStr">
+        <is>
+          <t>Wes noticed spacing issue while reviewing V12.</t>
         </is>
       </c>
     </row>
@@ -19003,6 +19088,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -19940,17 +20026,61 @@
       <c r="Z15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Opening ownership block</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Opening paragraphs / ownership listing</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Use trust sole-member sentence followed by four 4-character-indented authority lines.</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Apply BYH replacement as green text where new; preserve source strikethrough only where replacing source text.</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>First line normal block position; each later line starts with 4 spaces.</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Rule recorded for next build</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>Check line breaks and 4-character indentation after first line.</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>None currently.</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>R-022</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>BYH addition / formatting instruction</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>New BYH text green; indentation/line breaks are formatting rules.</t>
+        </is>
+      </c>
       <c r="L16" s="5" t="n"/>
       <c r="M16" s="5" t="n"/>
       <c r="N16" s="5" t="n"/>
@@ -19968,17 +20098,61 @@
       <c r="Z16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Opening agreement sentence</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Opening paragraph beginning parties hereto agree</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Correct entity replacement spacing so sentence reads cleanly as agreement of Buy Your Home, LLC.</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Do not allow source/replacement runs to join words; preserve proper spaces around stricken and added entity text.</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>No joined text such as ofSell Your Home, LLCBuy Your Home, LLC.</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Rule recorded for next build</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Search generated DOCX text for joined entity-name artifacts.</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>None currently.</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>R-023</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>BYH replacement spacing correction</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>New BYH replacement text green; source text keeps source formatting/strikethrough.</t>
+        </is>
+      </c>
       <c r="L17" s="5" t="n"/>
       <c r="M17" s="5" t="n"/>
       <c r="N17" s="5" t="n"/>
@@ -31256,7 +31430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z202"/>
+  <dimension ref="A1:Z204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -37310,6 +37484,78 @@
       <c r="X202" s="14" t="n"/>
       <c r="Y202" s="14" t="n"/>
       <c r="Z202" s="14" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B203" s="14" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="C203" s="14" t="inlineStr">
+        <is>
+          <t>Verify opening ownership block line breaks and 4-character indentation after the first line.</t>
+        </is>
+      </c>
+      <c r="D203" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E203" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F203" s="14" t="n"/>
+      <c r="G203" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H203" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-022.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B204" s="14" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="C204" s="14" t="inlineStr">
+        <is>
+          <t>Verify opening agreement sentence has proper spacing around Buy Your Home, LLC replacement and no joined ofSell/LLCBuy artifact.</t>
+        </is>
+      </c>
+      <c r="D204" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E204" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F204" s="14" t="n"/>
+      <c r="G204" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H204" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-023.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add BYH Exhibit A and certification exceptions
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -12629,7 +12629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z209"/>
+  <dimension ref="A1:Z212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12649,7 +12649,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -19049,6 +19048,132 @@
       <c r="H209" s="14" t="inlineStr">
         <is>
           <t>Wes noticed spacing issue while reviewing V12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="14" t="inlineStr">
+        <is>
+          <t>R-024</t>
+        </is>
+      </c>
+      <c r="B210" s="14" t="inlineStr">
+        <is>
+          <t>Exhibit A Completeness</t>
+        </is>
+      </c>
+      <c r="C210" s="14" t="inlineStr">
+        <is>
+          <t>Treat Exhibit A as incomplete until checked in the next build. Do not assume prior Exhibit A language fully states BYH sole-member, ownership, manager, trustee-authority, tax-classification, or signature requirements.</t>
+        </is>
+      </c>
+      <c r="D210" s="14" t="inlineStr">
+        <is>
+          <t>BYH Exhibit A</t>
+        </is>
+      </c>
+      <c r="E210" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F210" s="14" t="inlineStr">
+        <is>
+          <t>Requires Exhibit A completeness review before review-ready status</t>
+        </is>
+      </c>
+      <c r="G210" s="14" t="inlineStr">
+        <is>
+          <t>Compare Exhibit A against current BYH facts and User Inputs</t>
+        </is>
+      </c>
+      <c r="H210" s="14" t="inlineStr">
+        <is>
+          <t>Wes instruction on 2026-06-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="14" t="inlineStr">
+        <is>
+          <t>R-025</t>
+        </is>
+      </c>
+      <c r="B211" s="14" t="inlineStr">
+        <is>
+          <t>Certification Clean-Edit Exception</t>
+        </is>
+      </c>
+      <c r="C211" s="14" t="inlineStr">
+        <is>
+          <t>The certification/signature page is an exception to the normal history-preserving do-not-delete rule. Use clean edits without historical text that does not apply to BYH, and remove inapplicable certification/signature language rather than leaving confusing struck text.</t>
+        </is>
+      </c>
+      <c r="D211" s="14" t="inlineStr">
+        <is>
+          <t>Certification/signature page</t>
+        </is>
+      </c>
+      <c r="E211" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F211" s="14" t="inlineStr">
+        <is>
+          <t>Allows clean certification page instead of full redline history</t>
+        </is>
+      </c>
+      <c r="G211" s="14" t="inlineStr">
+        <is>
+          <t>Certification page contains only applicable signing language</t>
+        </is>
+      </c>
+      <c r="H211" s="14" t="inlineStr">
+        <is>
+          <t>Narrow exception; ordinary numbered sections still follow do-not-delete unless separately approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="14" t="inlineStr">
+        <is>
+          <t>R-026</t>
+        </is>
+      </c>
+      <c r="B212" s="14" t="inlineStr">
+        <is>
+          <t>Certification Effective Date</t>
+        </is>
+      </c>
+      <c r="C212" s="14" t="inlineStr">
+        <is>
+          <t>Correct the certification effective-date sentence in the next build. Do not leave 'on behalf of themselves and the Company, effective June ____, 2025' unless Wes confirms that exact date language; use the correct BYH effective date or flag as an open date issue.</t>
+        </is>
+      </c>
+      <c r="D212" s="14" t="inlineStr">
+        <is>
+          <t>Certification/signature page</t>
+        </is>
+      </c>
+      <c r="E212" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F212" s="14" t="inlineStr">
+        <is>
+          <t>Prevents stale 2025 blank-date language</t>
+        </is>
+      </c>
+      <c r="G212" s="14" t="inlineStr">
+        <is>
+          <t>Effective-date sentence is corrected or date issue is listed as open</t>
+        </is>
+      </c>
+      <c r="H212" s="14" t="inlineStr">
+        <is>
+          <t>Wes flagged stale date wording from V12.</t>
         </is>
       </c>
     </row>
@@ -19088,7 +19213,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -19954,59 +20078,59 @@
       <c r="Z14" s="5" t="n"/>
     </row>
     <row r="15" ht="38.25" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Exhibit A</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Member schedule</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Show Browning Family Revocable Trust as sole Member with 100 units / 100%; co-trustees as voting/signing authority.</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Strike prior retirement member table; add BYH table/rows in green.</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Preserve table/readability.</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Applied in V10+</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Exhibit text check.</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>Confirm address and trust details.</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>R-012</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>BYH addition / source strikeout as applicable</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>Preserve source colors; new BYH additions/replacements green.</t>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Exhibit A</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Review and complete Exhibit A for BYH sole-member, ownership, manager, trustee-authority, tax-classification, and signature requirements.</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Do not assume prior Exhibit A is complete; add missing BYH language in green or flag open issues.</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Preserve Exhibit A structure unless clean completion requires a clearer layout.</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Incomplete until checked in next build</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>Compare against current User Inputs and rule register before review-ready status.</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Confirm exact Exhibit A requirements for BYH if not fully determined.</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>R-024</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="inlineStr">
+        <is>
+          <t>BYH completion / open issue</t>
+        </is>
+      </c>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>New BYH language green; open unknowns flagged instead of guessed.</t>
         </is>
       </c>
       <c r="L15" s="5" t="n"/>
@@ -20170,17 +20294,61 @@
       <c r="Z17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Certification / signature page</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Certification and signature blocks</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Use clean applicable certification/signature language and correct the effective-date sentence.</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Clean-edit exception: remove inapplicable historical signing text instead of leaving confusing strikethrough on the certification page.</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Signing page should be clean and ready for review/signature, not a full historical redline page.</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Rule recorded for next build</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>No stale June ____, 2025 blank date unless expressly confirmed; only applicable signers/language shown.</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>BYH effective date must be confirmed or flagged open.</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>R-025, R-026</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>BYH clean-edit exception</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Clean certification page may omit historical struck text; new BYH text green where visible redline is still used.</t>
+        </is>
+      </c>
       <c r="L18" s="5" t="n"/>
       <c r="M18" s="5" t="n"/>
       <c r="N18" s="5" t="n"/>
@@ -26069,14 +26237,46 @@
       <c r="Z9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>OI-EFFDATE-001</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Confirm the correct BYH certification effective date; do not leave June ____, 2025 unless Wes confirms it.</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Effective date is open until confirmed.</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Wes / attorney or CPA as needed</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Added from Wes instruction on 2026-06-08; controlled by R-026.</t>
+        </is>
+      </c>
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
       <c r="K10" s="5" t="n"/>
@@ -31430,7 +31630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z204"/>
+  <dimension ref="A1:Z207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -31450,7 +31650,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -37554,6 +37753,114 @@
       <c r="H204" s="14" t="inlineStr">
         <is>
           <t>Rule R-023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="B205" s="14" t="inlineStr">
+        <is>
+          <t>Exhibit A</t>
+        </is>
+      </c>
+      <c r="C205" s="14" t="inlineStr">
+        <is>
+          <t>Check Exhibit A for completeness against BYH sole-member, ownership, manager, trustee-authority, tax-classification, and signature requirements.</t>
+        </is>
+      </c>
+      <c r="D205" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E205" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F205" s="14" t="n"/>
+      <c r="G205" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H205" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B206" s="14" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="C206" s="14" t="inlineStr">
+        <is>
+          <t>Apply clean-edit exception on certification/signature page; remove inapplicable historical text instead of leaving confusing strike-through.</t>
+        </is>
+      </c>
+      <c r="D206" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E206" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F206" s="14" t="n"/>
+      <c r="G206" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H206" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="B207" s="14" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="C207" s="14" t="inlineStr">
+        <is>
+          <t>Correct or flag the certification effective-date sentence; do not leave June ____, 2025 unless Wes confirms it.</t>
+        </is>
+      </c>
+      <c r="D207" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E207" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F207" s="14" t="n"/>
+      <c r="G207" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H207" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Define BYH Exhibit A and signature block cleanup
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -12629,7 +12629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z212"/>
+  <dimension ref="A1:Z214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12649,6 +12649,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -19174,6 +19175,90 @@
       <c r="H212" s="14" t="inlineStr">
         <is>
           <t>Wes flagged stale date wording from V12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="14" t="inlineStr">
+        <is>
+          <t>R-027</t>
+        </is>
+      </c>
+      <c r="B213" s="14" t="inlineStr">
+        <is>
+          <t>Clean Exhibit A Member List</t>
+        </is>
+      </c>
+      <c r="C213" s="14" t="inlineStr">
+        <is>
+          <t>Exhibit A should be clean for BYH and should show only the new/current BYH member information. Do not leave old member information or historical source text on the Exhibit A page.</t>
+        </is>
+      </c>
+      <c r="D213" s="14" t="inlineStr">
+        <is>
+          <t>BYH Exhibit A</t>
+        </is>
+      </c>
+      <c r="E213" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F213" s="14" t="inlineStr">
+        <is>
+          <t>Creates clean BYH Exhibit A instead of historical redline exhibit</t>
+        </is>
+      </c>
+      <c r="G213" s="14" t="inlineStr">
+        <is>
+          <t>Exhibit A has only current BYH member information and no old member text</t>
+        </is>
+      </c>
+      <c r="H213" s="14" t="inlineStr">
+        <is>
+          <t>Wes instruction on 2026-06-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="14" t="inlineStr">
+        <is>
+          <t>R-028</t>
+        </is>
+      </c>
+      <c r="B214" s="14" t="inlineStr">
+        <is>
+          <t>Defined Signature Blocks</t>
+        </is>
+      </c>
+      <c r="C214" s="14" t="inlineStr">
+        <is>
+          <t>Signature blocks should be more defined per person or entity. Keep line spacing tighter inside each signer group, and use more vertical space between separate signer groups so Wesley Dale Browning, Jeanette Wilson Hollinger, and Investment Services LLC appear as distinct signing groups.</t>
+        </is>
+      </c>
+      <c r="D214" s="14" t="inlineStr">
+        <is>
+          <t>Certification/signature page</t>
+        </is>
+      </c>
+      <c r="E214" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F214" s="14" t="inlineStr">
+        <is>
+          <t>Improves signature page readability and avoids grouping signers together</t>
+        </is>
+      </c>
+      <c r="G214" s="14" t="inlineStr">
+        <is>
+          <t>Each signer group is visually distinct, with tighter intra-group spacing and more inter-group space</t>
+        </is>
+      </c>
+      <c r="H214" s="14" t="inlineStr">
+        <is>
+          <t>Works with certification clean-edit exception R-025.</t>
         </is>
       </c>
     </row>
@@ -20090,17 +20175,17 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Review and complete Exhibit A for BYH sole-member, ownership, manager, trustee-authority, tax-classification, and signature requirements.</t>
+          <t>Review and complete Exhibit A with only current BYH member information; remove old member information and historical source text.</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Do not assume prior Exhibit A is complete; add missing BYH language in green or flag open issues.</t>
+          <t>Clean Exhibit A exception: do not leave old member information struck through on the Exhibit A page.</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>Preserve Exhibit A structure unless clean completion requires a clearer layout.</t>
+          <t>Clean BYH exhibit; preserve useful exhibit structure but omit historical source clutter.</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
@@ -20110,27 +20195,27 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Compare against current User Inputs and rule register before review-ready status.</t>
+          <t>Exhibit A shows only current BYH member information and passes completeness review.</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>Confirm exact Exhibit A requirements for BYH if not fully determined.</t>
+          <t>Confirm exact final Exhibit A member details and any required tax/manager fields.</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>R-024</t>
+          <t>R-024, R-027</t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>BYH completion / open issue</t>
+          <t>BYH clean Exhibit A</t>
         </is>
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>New BYH language green; open unknowns flagged instead of guessed.</t>
+          <t>Clean exhibit may omit historical struck text; use green only for visible new BYH drafting if needed.</t>
         </is>
       </c>
       <c r="L15" s="5" t="n"/>
@@ -20306,7 +20391,7 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Use clean applicable certification/signature language and correct the effective-date sentence.</t>
+          <t>Use clean applicable certification/signature language, correct the effective-date sentence, and create defined signer blocks per person/entity.</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
@@ -20316,7 +20401,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Signing page should be clean and ready for review/signature, not a full historical redline page.</t>
+          <t>Tighter line spacing inside each signer group; more vertical space between Wesley Dale Browning, Jeanette Wilson Hollinger, and Investment Services LLC groups.</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -20326,17 +20411,17 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>No stale June ____, 2025 blank date unless expressly confirmed; only applicable signers/language shown.</t>
+          <t>Each signer group is visually distinct and no signer is grouped with another by layout accident.</t>
         </is>
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>BYH effective date must be confirmed or flagged open.</t>
+          <t>BYH effective date and Investment Services LLC signer/title must be confirmed or flagged open.</t>
         </is>
       </c>
       <c r="I18" s="14" t="inlineStr">
         <is>
-          <t>R-025, R-026</t>
+          <t>R-025, R-026, R-028</t>
         </is>
       </c>
       <c r="J18" s="14" t="inlineStr">
@@ -31630,7 +31715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z207"/>
+  <dimension ref="A1:Z209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.75" customWidth="1" min="1" max="1"/>
@@ -31650,6 +31735,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -37861,6 +37947,78 @@
       <c r="H207" s="14" t="inlineStr">
         <is>
           <t>Rule R-026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="B208" s="14" t="inlineStr">
+        <is>
+          <t>Exhibit A</t>
+        </is>
+      </c>
+      <c r="C208" s="14" t="inlineStr">
+        <is>
+          <t>Verify Exhibit A is clean for BYH and contains only current BYH member information, with no old member text.</t>
+        </is>
+      </c>
+      <c r="D208" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E208" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F208" s="14" t="n"/>
+      <c r="G208" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H208" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="14" t="n">
+        <v>23</v>
+      </c>
+      <c r="B209" s="14" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="C209" s="14" t="inlineStr">
+        <is>
+          <t>Verify signature blocks are defined per person/entity, with tighter spacing inside groups and more space between groups.</t>
+        </is>
+      </c>
+      <c r="D209" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E209" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F209" s="14" t="n"/>
+      <c r="G209" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H209" s="14" t="inlineStr">
+        <is>
+          <t>Rule R-028.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build BYH OA V13 draft
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -7400,49 +7400,49 @@
       <c r="Z15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>V13</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>V13 - BYH OA Draft ...</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Simplified OA refreshed from Teams</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Future fresh cumulative</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Use version-first filename and workbook-controlled rules</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>V13 - BYH OA Draft Clean Certification and Exhibit A - from Simplified OA.docx</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Simplified OA local refreshed copy</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Fresh cumulative</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Green BYH additions, opening block indentation, clean certification page, clean Exhibit A</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Jeff red/BYH color separation; stale certification date; old Exhibit A member text; signature block grouping</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>Current review draft</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>V13 - BYH OA vs V12 Comparison.md; V13 notes file</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="inlineStr">
+        <is>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -12649,7 +12649,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -25901,6 +25900,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -26382,14 +26382,46 @@
       <c r="Z10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>OI-SRCREFRESH-001</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Source refresh</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>V13 used the local refreshed Simplified OA because Teams/SharePoint refresh was not available in this tool session.</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Local Simplified OA is the latest available source copy in the project room.</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Codex / Wes</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>Before final legal draft</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>Refresh from Teams before treating a later build as final if Teams source may have changed.</t>
+        </is>
+      </c>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
@@ -31735,7 +31767,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Build BYH OA V14 observation fixes
</commit_message>
<xml_diff>
--- a/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
+++ b/Project Rooms/Operating Agreements/working/BYH OA Process Control.xlsx
@@ -7432,7 +7432,7 @@
       </c>
       <c r="G16" s="19" t="inlineStr">
         <is>
-          <t>Current review draft</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="H16" s="19" t="inlineStr">
@@ -7442,7 +7442,7 @@
       </c>
       <c r="I16" s="19" t="inlineStr">
         <is>
-          <t>Candidate</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -7464,15 +7464,51 @@
       <c r="Z16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>V14</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>V14 - BYH OA Draft Observation Fixes - from Simplified OA.docx</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Simplified OA local refreshed copy</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Fresh cumulative</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>Observation fixes: opening agreement spacing, Article 2 2.1(d), 5.1(b)(xi) retained, and 9.5 mostly retained with only the retirement guarantee sentence struck.</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Corrects unnumbered Article 2 insertion, joined entity-name spacing artifact, and overbroad 9.5 strikeout.</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>Current review draft</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>V14 - BYH OA vs V13 Comparison.md; V14 notes file</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
       <c r="J17" s="5" t="n"/>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="5" t="n"/>
@@ -13550,14 +13586,46 @@
       <c r="Z17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>R-029</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Article 2 Numbering</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>For BYH, add the sole-member and co-trustee voting authority provision as Section 2.1(d), not as an unnumbered paragraph and not as a replacement for existing 2.1.</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Article 2</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Keeps the new trust voting concept anchored without disturbing existing enumeration.</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Check for 2.1(d) heading/text and absence of duplicate unnumbered sole-member paragraph.</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Wes instruction on 2026-06-08.</t>
+        </is>
+      </c>
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
       <c r="K18" s="5" t="n"/>
@@ -13578,14 +13646,46 @@
       <c r="Z18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="9" t="n"/>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>R-030</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Section 9.5 Borrowing Money</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>For BYH, leave Section 9.5 Borrowing Money operative except strike only the final retirement-account/disqualified-person guarantee sentence.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Section 9.5</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Keeps useful borrowing authority while removing retirement-account restriction language that does not apply to BYH.</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Check 9.5 first sentence is unstruck and final sentence beginning However, Members described in Section 9.1 is struck.</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Wes approved this treatment on 2026-06-08.</t>
+        </is>
+      </c>
       <c r="I19" s="5" t="n"/>
       <c r="J19" s="5" t="n"/>
       <c r="K19" s="5" t="n"/>
@@ -13606,14 +13706,46 @@
       <c r="Z19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>R-031</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Future Final Clean Version</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>When a review draft is promoted to a final clean version, remove partial word or phrase strikeouts and retain only whole struck numbered clauses where needed to preserve enumeration or cross-reference integrity.</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Final clean BYH versions</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Active for finalization</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Separates review-history preservation from final-form readability.</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Final clean pass checks for partial strike remnants and preserved whole numbered clauses only where intentionally retained.</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Do not apply automatically to review drafts unless Wes asks for a final clean version.</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="n"/>
       <c r="J20" s="5" t="n"/>
       <c r="K20" s="5" t="n"/>
@@ -19613,7 +19745,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Applied in V12</t>
+          <t>Superseded by V14 placement rule</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -19623,7 +19755,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Confirm whether paragraph should be numbered or unnumbered in final legal drafting.</t>
+          <t>V14 uses numbered 2.1(d) placement instead of an unnumbered insertion.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -19973,12 +20105,12 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Rule recorded for next build</t>
+          <t>Applied in V14</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>Confirm 5.1(b)(xi) appears unstruck in the next review-ready BYH draft.</t>
+          <t>V14 structural check confirms 5.1(b)(xi) is present and unstruck.</t>
         </is>
       </c>
       <c r="H12" s="19" t="inlineStr">
@@ -20189,7 +20321,7 @@
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Incomplete until checked in next build</t>
+          <t>Applied in V13 and retained in V14</t>
         </is>
       </c>
       <c r="G15" s="19" t="inlineStr">
@@ -20333,12 +20465,12 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Rule recorded for next build</t>
+          <t>Applied in V14</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>Search generated DOCX text for joined entity-name artifacts.</t>
+          <t>Structural text check confirms no joined ofSell/LLCBuy artifact; visible spacing preserved around source and BYH entity names.</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
@@ -20405,7 +20537,7 @@
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Rule recorded for next build</t>
+          <t>Applied in V13 and retained in V14</t>
         </is>
       </c>
       <c r="G18" s="14" t="inlineStr">
@@ -20450,16 +20582,56 @@
       <c r="Z18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>2.1(d) Sole Member and Voting Authority</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Article 2 after Description of the Membership Units</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Add the BYH sole-member/co-trustee voting authority as numbered 2.1(d).</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Add green BYH paragraph; do not strike existing 2.1 and do not use unnumbered lead-in text.</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Preserve article structure; avoid article-title lead-in.</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Applied in V14</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>2.1(d) present; unnumbered sole-member paragraph absent.</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>Confirm final legal wording with counsel before final clean version.</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t>R-005, R-006, R-012, R-029</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>BYH addition</t>
+        </is>
+      </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="5" t="n"/>
       <c r="M19" s="5" t="n"/>
@@ -20478,16 +20650,56 @@
       <c r="Z19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>9.5 Borrowing Money</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Section 9.5</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Retain borrowing authority but remove retirement-account guarantee restriction that does not apply to BYH.</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Keep first sentence unstruck; strike only final retirement/disqualified-person guarantee sentence.</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Minimal partial strike only for review draft; final-clean rule may remove partial strike later.</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Applied in V14</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>9.5 first sentence unstruck; final sentence struck.</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>Legal review of borrowing authority still required.</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="inlineStr">
+        <is>
+          <t>R-004, R-005, R-030, R-031</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="inlineStr">
+        <is>
+          <t>Source retained / BYH strikeout</t>
+        </is>
+      </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="5" t="n"/>
       <c r="M20" s="5" t="n"/>
@@ -20506,16 +20718,56 @@
       <c r="Z20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Final clean strikeout treatment</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Future final clean version</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Remove partial strikeouts when promoting a draft to final form; preserve only whole struck numbered clauses where needed to protect enumeration/cross-references.</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Final-clean exception, not automatic review-draft behavior.</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Clean final text while preserving numbering where needed.</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Rule recorded for future finalization</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>Final clean pass checks for partial strikes and retained whole numbered clauses.</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>Wait for Wes to request final clean version.</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>R-031</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>Finalization rule</t>
+        </is>
+      </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="5" t="n"/>
       <c r="M21" s="5" t="n"/>
@@ -25900,7 +26152,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -31848,10 +32099,14 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Pending for next build</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="n"/>
+          <t>Complete for V14</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Wes said go after observation list.</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>Wes</t>
@@ -31902,10 +32157,14 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n"/>
+          <t>Not refreshed this run</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>V14 used the existing local refreshed Simplified OA source from the prior fresh-build process.</t>
+        </is>
+      </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -31956,10 +32215,14 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n"/>
+          <t>Complete for V14</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Rules R-001 through R-031 considered.</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -32010,10 +32273,14 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="n"/>
+          <t>Complete for V14</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>V14 builder uses Simplified OA source, not V13 as its draft source.</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -32442,10 +32709,14 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n"/>
+          <t>Structural complete; visual render pending/unavailable</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Structural checks passed; visual converter availability checked separately.</t>
+        </is>
+      </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -32496,10 +32767,14 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n"/>
+          <t>Complete for V14</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>V14 notes, comparison, README, source inventory, and workbook updated.</t>
+        </is>
+      </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -32550,10 +32825,14 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n"/>
+          <t>Pending commit</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Commit after final review of V14 package.</t>
+        </is>
+      </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
           <t>Codex</t>
@@ -32584,14 +32863,44 @@
       <c r="Z17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
+      <c r="A18" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Article 2</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Verify sole-member/trustee voting provision is numbered 2.1(d).</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Complete for V14</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>DOCX structural check: 2.1(d) present; unnumbered sole-member paragraph absent.</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Rule R-029.</t>
+        </is>
+      </c>
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
       <c r="K18" s="5" t="n"/>
@@ -32612,14 +32921,44 @@
       <c r="Z18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="9" t="n"/>
+      <c r="A19" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Verify 9.5 Borrowing Money is retained except final retirement-account guarantee sentence.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Complete for V14</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>DOCX run check: first 9.5 sentence unstruck; final sentence struck.</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Rule R-030.</t>
+        </is>
+      </c>
       <c r="I19" s="5" t="n"/>
       <c r="J19" s="5" t="n"/>
       <c r="K19" s="5" t="n"/>
@@ -32640,14 +32979,44 @@
       <c r="Z19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
+      <c r="A20" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Finalization</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Do not clean partial strikeouts until Wes asks to promote a draft to final clean version.</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Rule recorded</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Rule R-031 added to Rule Register and Article Map.</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Codex/Wes</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Review drafts continue to show redline history unless instructed otherwise.</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="n"/>
       <c r="J20" s="5" t="n"/>
       <c r="K20" s="5" t="n"/>

</xml_diff>